<commit_message>
Modified each model to save out put to /data/tmp/ folder, added input_out functions for that, added a script for comparison plot
</commit_message>
<xml_diff>
--- a/data/data_clean.xlsx
+++ b/data/data_clean.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/73d4a18d9c9284b4/KULeuven/Ac2Gen/preDissemination/Acetate-Acrylate_review/ML_Literature/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_5EF5D0B7D320D16E5FF93111595ED87656C52FEA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_5EF5D0B7D320D16E5FF93111595ED87656C52FEA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{575ECCE8-02EC-470F-979D-216DCEF909C2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -793,6 +793,53 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AW315"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="2.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="3.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="2.28515625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="3" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="12" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="43.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>